<commit_message>
Updated the test cases file
</commit_message>
<xml_diff>
--- a/doc/coinmarketcap-test cases.xlsx
+++ b/doc/coinmarketcap-test cases.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30128"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{124F771B-2CD2-440E-A30D-E4DD8461903D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{99CBA38C-4FBE-4D41-BF6D-1F2F71B932C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="WF1 - Search" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="264" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="267" uniqueCount="158">
   <si>
     <t>TC ID</t>
   </si>
@@ -357,6 +357,9 @@
     <t>The converted result is 0 / handled with no error</t>
   </si>
   <si>
+    <t>The converter is stuck in a infinite loop animation</t>
+  </si>
+  <si>
     <t>FAIL</t>
   </si>
   <si>
@@ -404,7 +407,7 @@
     <t>TC_CC_12</t>
   </si>
   <si>
-    <t>Enter two plus Befire a number for the amount</t>
+    <t>Enter two plus Before the number</t>
   </si>
   <si>
     <t>1. Set From = BTC
@@ -420,6 +423,9 @@
     <t>The convertor should ingore the extra plus and calute the +5 amount</t>
   </si>
   <si>
+    <t>The converter didn't update with the value it is stuch on 1(the default value)</t>
+  </si>
+  <si>
     <t>TC_SF_01</t>
   </si>
   <si>
@@ -549,7 +555,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -578,11 +584,6 @@
     </font>
     <font>
       <sz val="10"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
     </font>
@@ -759,7 +760,7 @@
     <xf numFmtId="0" fontId="3" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -774,17 +775,17 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1424,7 +1425,7 @@
     <col min="4" max="4" width="33" customWidth="1"/>
     <col min="5" max="5" width="16.7109375" customWidth="1"/>
     <col min="6" max="6" width="28.7109375" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" customWidth="1"/>
+    <col min="7" max="7" width="22.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="28.5">
@@ -1475,7 +1476,7 @@
       <c r="F2" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="G2" s="25" t="s">
+      <c r="G2" s="24" t="s">
         <v>15</v>
       </c>
       <c r="H2" s="14" t="s">
@@ -1504,7 +1505,7 @@
       <c r="F3" s="12" t="s">
         <v>66</v>
       </c>
-      <c r="G3" s="25" t="s">
+      <c r="G3" s="24" t="s">
         <v>15</v>
       </c>
       <c r="H3" s="14" t="s">
@@ -1533,7 +1534,7 @@
       <c r="F4" s="12" t="s">
         <v>71</v>
       </c>
-      <c r="G4" s="25" t="s">
+      <c r="G4" s="24" t="s">
         <v>15</v>
       </c>
       <c r="H4" s="14" t="s">
@@ -1562,7 +1563,7 @@
       <c r="F5" s="12" t="s">
         <v>77</v>
       </c>
-      <c r="G5" s="25" t="s">
+      <c r="G5" s="24" t="s">
         <v>15</v>
       </c>
       <c r="H5" s="14" t="s">
@@ -1591,7 +1592,7 @@
       <c r="F6" s="12" t="s">
         <v>82</v>
       </c>
-      <c r="G6" s="25" t="s">
+      <c r="G6" s="24" t="s">
         <v>15</v>
       </c>
       <c r="H6" s="14" t="s">
@@ -1620,7 +1621,7 @@
       <c r="F7" s="12" t="s">
         <v>87</v>
       </c>
-      <c r="G7" s="25" t="s">
+      <c r="G7" s="24" t="s">
         <v>15</v>
       </c>
       <c r="H7" s="14" t="s">
@@ -1649,7 +1650,7 @@
       <c r="F8" s="12" t="s">
         <v>92</v>
       </c>
-      <c r="G8" s="25" t="s">
+      <c r="G8" s="24" t="s">
         <v>15</v>
       </c>
       <c r="H8" s="14" t="s">
@@ -1659,7 +1660,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="36">
+    <row r="9" spans="1:9" ht="39" customHeight="1">
       <c r="A9" s="12" t="s">
         <v>93</v>
       </c>
@@ -1678,61 +1679,65 @@
       <c r="F9" s="12" t="s">
         <v>97</v>
       </c>
-      <c r="G9" s="25"/>
+      <c r="G9" s="25" t="s">
+        <v>98</v>
+      </c>
       <c r="H9" s="14" t="s">
         <v>16</v>
       </c>
       <c r="I9" s="16" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" ht="36">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="33" customHeight="1">
       <c r="A10" s="12" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B10" s="12" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C10" s="12" t="s">
         <v>63</v>
       </c>
       <c r="D10" s="13" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="E10" s="12">
         <v>-1</v>
       </c>
       <c r="F10" s="12" t="s">
-        <v>102</v>
-      </c>
-      <c r="G10" s="25"/>
+        <v>103</v>
+      </c>
+      <c r="G10" s="25" t="s">
+        <v>98</v>
+      </c>
       <c r="H10" s="14" t="s">
         <v>16</v>
       </c>
       <c r="I10" s="16" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="24">
       <c r="A11" s="12" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B11" s="12" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C11" s="12" t="s">
         <v>63</v>
       </c>
       <c r="D11" s="13" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="E11" s="12" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="F11" s="12" t="s">
-        <v>107</v>
-      </c>
-      <c r="G11" s="25" t="s">
+        <v>108</v>
+      </c>
+      <c r="G11" s="24" t="s">
         <v>15</v>
       </c>
       <c r="H11" s="14" t="s">
@@ -1744,24 +1749,24 @@
     </row>
     <row r="12" spans="1:9" ht="24">
       <c r="A12" s="12" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B12" s="12" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C12" s="12" t="s">
         <v>63</v>
       </c>
       <c r="D12" s="13" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="E12" s="12" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="F12" s="12" t="s">
-        <v>107</v>
-      </c>
-      <c r="G12" s="25" t="s">
+        <v>108</v>
+      </c>
+      <c r="G12" s="24" t="s">
         <v>15</v>
       </c>
       <c r="H12" s="14" t="s">
@@ -1773,29 +1778,31 @@
     </row>
     <row r="13" spans="1:9" ht="60">
       <c r="A13" s="12" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B13" s="19" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C13" s="18" t="s">
         <v>63</v>
       </c>
       <c r="D13" s="20" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="E13" s="21" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="F13" s="22" t="s">
-        <v>116</v>
-      </c>
-      <c r="G13" s="23"/>
+        <v>117</v>
+      </c>
+      <c r="G13" s="19" t="s">
+        <v>118</v>
+      </c>
       <c r="H13" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="I13" s="24" t="s">
-        <v>98</v>
+      <c r="I13" s="23" t="s">
+        <v>99</v>
       </c>
     </row>
   </sheetData>
@@ -1844,19 +1851,19 @@
     </row>
     <row r="2" spans="1:8" ht="24">
       <c r="A2" s="6" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="D2" s="10" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="E2" s="9" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="F2" s="1"/>
       <c r="G2" s="8" t="s">
@@ -1866,19 +1873,19 @@
     </row>
     <row r="3" spans="1:8" ht="24">
       <c r="A3" s="6" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="D3" s="10" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="F3" s="1"/>
       <c r="G3" s="8" t="s">
@@ -1888,19 +1895,19 @@
     </row>
     <row r="4" spans="1:8" ht="36">
       <c r="A4" s="6" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="F4" s="1"/>
       <c r="G4" s="8" t="s">
@@ -1910,19 +1917,19 @@
     </row>
     <row r="5" spans="1:8" ht="48">
       <c r="A5" s="6" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="F5" s="1"/>
       <c r="G5" s="8" t="s">
@@ -1932,19 +1939,19 @@
     </row>
     <row r="6" spans="1:8" ht="24">
       <c r="A6" s="6" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="D6" s="10" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="F6" s="1"/>
       <c r="G6" s="8" t="s">
@@ -1954,19 +1961,19 @@
     </row>
     <row r="7" spans="1:8" ht="24">
       <c r="A7" s="6" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="D7" s="10" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F7" s="1"/>
       <c r="G7" s="8" t="s">
@@ -1976,19 +1983,19 @@
     </row>
     <row r="8" spans="1:8" ht="24">
       <c r="A8" s="6" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="D8" s="10" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="F8" s="1"/>
       <c r="G8" s="8" t="s">
@@ -1998,19 +2005,19 @@
     </row>
     <row r="9" spans="1:8" ht="24">
       <c r="A9" s="6" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="C9" s="9" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="D9" s="10" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="F9" s="1"/>
       <c r="G9" s="8" t="s">
@@ -2020,19 +2027,19 @@
     </row>
     <row r="10" spans="1:8" ht="36">
       <c r="A10" s="6" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="D10" s="10" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="F10" s="1"/>
       <c r="G10" s="8" t="s">

</xml_diff>

<commit_message>
removed wf3 from the doc
</commit_message>
<xml_diff>
--- a/doc/coinmarketcap-test cases.xlsx
+++ b/doc/coinmarketcap-test cases.xlsx
@@ -1,16 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30128"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{99CBA38C-4FBE-4D41-BF6D-1F2F71B932C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ASUS\eclipse-workspace\coinmarketcap\doc\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B66A47C-C152-496A-9BDD-BEB5F6B77715}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="WF1 - Search" sheetId="1" r:id="rId1"/>
     <sheet name="WF2 -  Converter" sheetId="2" r:id="rId2"/>
-    <sheet name="WF 3 - coin table order " sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -33,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="267" uniqueCount="158">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="119">
   <si>
     <t>TC ID</t>
   </si>
@@ -425,137 +429,12 @@
   <si>
     <t>The converter didn't update with the value it is stuch on 1(the default value)</t>
   </si>
-  <si>
-    <t>TC_SF_01</t>
-  </si>
-  <si>
-    <t>Default table ordering</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> All-coins table is loaded</t>
-  </si>
-  <si>
-    <t>1. Open the main coin listings table</t>
-  </si>
-  <si>
-    <t>Coins are listed by rank (market cap), starting at 1, 2, 3 …</t>
-  </si>
-  <si>
-    <t>TC_SF_02</t>
-  </si>
-  <si>
-    <t>Sort by Volume ascending</t>
-  </si>
-  <si>
-    <t>Coin table is loaded</t>
-  </si>
-  <si>
-    <t>1. Click the “Price” column header</t>
-  </si>
-  <si>
-    <t>Rows are reordered with prices from lowest to highest</t>
-  </si>
-  <si>
-    <t>TC_SF_03</t>
-  </si>
-  <si>
-    <t>Sort by Volume descending</t>
-  </si>
-  <si>
-    <t>1. Click the “Price” column header
-2. Click the "Price" column header again</t>
-  </si>
-  <si>
-    <t>Rows are reordered with prices from highest to lowest</t>
-  </si>
-  <si>
-    <t>TC_SF_04</t>
-  </si>
-  <si>
-    <t>Sort by Market Cap</t>
-  </si>
-  <si>
-    <t>1. Click the “Market Cap” column header
-2. Click the "Market Cap" column header again</t>
-  </si>
-  <si>
-    <t>Rows are reordered according to market cap in the chosen direction</t>
-  </si>
-  <si>
-    <t>TC_SF_05</t>
-  </si>
-  <si>
-    <t>Navigate to the next page</t>
-  </si>
-  <si>
-    <t>1. Scroll to pagination
-2. Click “Next”</t>
-  </si>
-  <si>
-    <t>A new set of coins (ranks continuing from previous page) is displayed</t>
-  </si>
-  <si>
-    <t>TC_SF_06</t>
-  </si>
-  <si>
-    <t>Jump to a specific page number</t>
-  </si>
-  <si>
-    <t>1. Click a specific page number (e.g. 3)</t>
-  </si>
-  <si>
-    <t>The table shows the coins belonging to that page</t>
-  </si>
-  <si>
-    <t>TC_SF_07</t>
-  </si>
-  <si>
-    <t>Change rows per page</t>
-  </si>
-  <si>
-    <t>1. Open rows-per-page control
-2. Select 300</t>
-  </si>
-  <si>
-    <t>The table displays the selected number of rows</t>
-  </si>
-  <si>
-    <t>TC_SF_08</t>
-  </si>
-  <si>
-    <t>Pagination boundary on last page</t>
-  </si>
-  <si>
-    <t>On the last available page</t>
-  </si>
-  <si>
-    <t>1. Navigate to the last page
-2. Attempt to click “Next”</t>
-  </si>
-  <si>
-    <t>The “Next” control is disabled / no further page loads</t>
-  </si>
-  <si>
-    <t>TC_SF_09</t>
-  </si>
-  <si>
-    <t>Set layout to Top Gainers</t>
-  </si>
-  <si>
-    <t>1. Click Colums button
-2. Click on the drop down meun
-3. Select Top Gainers</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Coins are listed by rank (market cap), starting at 1, 2, 3 …
-</t>
-  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -710,7 +589,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment readingOrder="1"/>
@@ -735,12 +614,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
@@ -1107,19 +980,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I10"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="10.5703125" customWidth="1"/>
-    <col min="2" max="2" width="37.140625" customWidth="1"/>
-    <col min="3" max="3" width="17.5703125" customWidth="1"/>
-    <col min="4" max="4" width="39.140625" customWidth="1"/>
+    <col min="1" max="1" width="10.5546875" customWidth="1"/>
+    <col min="2" max="2" width="37.109375" customWidth="1"/>
+    <col min="3" max="3" width="17.5546875" customWidth="1"/>
+    <col min="4" max="4" width="39.109375" customWidth="1"/>
     <col min="5" max="5" width="15" customWidth="1"/>
-    <col min="6" max="6" width="39.42578125" customWidth="1"/>
-    <col min="7" max="8" width="13.42578125" customWidth="1"/>
-    <col min="9" max="9" width="7.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="39.44140625" customWidth="1"/>
+    <col min="7" max="8" width="13.44140625" customWidth="1"/>
+    <col min="9" max="9" width="7.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="28.5">
+    <row r="1" spans="1:9" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -1148,7 +1021,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="36">
+    <row r="2" spans="1:9" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A2" s="6" t="s">
         <v>9</v>
       </c>
@@ -1177,7 +1050,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="36">
+    <row r="3" spans="1:9" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A3" s="6" t="s">
         <v>18</v>
       </c>
@@ -1206,7 +1079,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="36">
+    <row r="4" spans="1:9" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A4" s="6" t="s">
         <v>23</v>
       </c>
@@ -1235,7 +1108,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="24">
+    <row r="5" spans="1:9" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A5" s="6" t="s">
         <v>28</v>
       </c>
@@ -1264,7 +1137,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="24">
+    <row r="6" spans="1:9" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A6" s="6" t="s">
         <v>33</v>
       </c>
@@ -1293,7 +1166,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="24">
+    <row r="7" spans="1:9" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A7" s="6" t="s">
         <v>38</v>
       </c>
@@ -1322,7 +1195,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="24">
+    <row r="8" spans="1:9" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A8" s="6" t="s">
         <v>43</v>
       </c>
@@ -1351,7 +1224,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="24">
+    <row r="9" spans="1:9" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A9" s="6" t="s">
         <v>47</v>
       </c>
@@ -1380,7 +1253,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="24">
+    <row r="10" spans="1:9" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A10" s="6" t="s">
         <v>50</v>
       </c>
@@ -1417,635 +1290,393 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D40200E8-913F-4058-BFEA-0BEB482B3B00}">
   <dimension ref="A1:I13"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12.42578125" customWidth="1"/>
-    <col min="2" max="2" width="29.85546875" customWidth="1"/>
-    <col min="3" max="3" width="24.5703125" customWidth="1"/>
+    <col min="1" max="1" width="12.44140625" customWidth="1"/>
+    <col min="2" max="2" width="29.88671875" customWidth="1"/>
+    <col min="3" max="3" width="24.5546875" customWidth="1"/>
     <col min="4" max="4" width="33" customWidth="1"/>
-    <col min="5" max="5" width="16.7109375" customWidth="1"/>
-    <col min="6" max="6" width="28.7109375" customWidth="1"/>
-    <col min="7" max="7" width="22.7109375" customWidth="1"/>
+    <col min="5" max="5" width="16.6640625" customWidth="1"/>
+    <col min="6" max="6" width="28.6640625" customWidth="1"/>
+    <col min="7" max="7" width="22.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="28.5">
-      <c r="A1" s="11" t="s">
+    <row r="1" spans="1:9" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="11" t="s">
+      <c r="B1" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="11" t="s">
+      <c r="C1" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="11" t="s">
+      <c r="D1" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="11" t="s">
+      <c r="E1" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="11" t="s">
+      <c r="F1" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="11" t="s">
+      <c r="G1" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="11" t="s">
+      <c r="H1" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="11" t="s">
+      <c r="I1" s="9" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="36">
-      <c r="A2" s="12" t="s">
+    <row r="2" spans="1:9" ht="39.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="B2" s="12" t="s">
+      <c r="B2" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="C2" s="12" t="s">
+      <c r="C2" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="D2" s="13" t="s">
+      <c r="D2" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="E2" s="12" t="s">
+      <c r="E2" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="F2" s="12" t="s">
+      <c r="F2" s="10" t="s">
         <v>60</v>
       </c>
-      <c r="G2" s="24" t="s">
-        <v>15</v>
-      </c>
-      <c r="H2" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="I2" s="15" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" ht="36">
-      <c r="A3" s="12" t="s">
+      <c r="G2" s="22" t="s">
+        <v>15</v>
+      </c>
+      <c r="H2" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="I2" s="13" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" ht="39.6" x14ac:dyDescent="0.3">
+      <c r="A3" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="B3" s="12" t="s">
+      <c r="B3" s="10" t="s">
         <v>62</v>
       </c>
-      <c r="C3" s="12" t="s">
+      <c r="C3" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="D3" s="13" t="s">
+      <c r="D3" s="11" t="s">
         <v>64</v>
       </c>
-      <c r="E3" s="12" t="s">
+      <c r="E3" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="F3" s="12" t="s">
+      <c r="F3" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="G3" s="24" t="s">
-        <v>15</v>
-      </c>
-      <c r="H3" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="I3" s="15" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" ht="36">
-      <c r="A4" s="12" t="s">
+      <c r="G3" s="22" t="s">
+        <v>15</v>
+      </c>
+      <c r="H3" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="I3" s="13" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" ht="39.6" x14ac:dyDescent="0.3">
+      <c r="A4" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="B4" s="12" t="s">
+      <c r="B4" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="C4" s="12" t="s">
+      <c r="C4" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="D4" s="13" t="s">
+      <c r="D4" s="11" t="s">
         <v>69</v>
       </c>
-      <c r="E4" s="12" t="s">
+      <c r="E4" s="10" t="s">
         <v>70</v>
       </c>
-      <c r="F4" s="12" t="s">
+      <c r="F4" s="10" t="s">
         <v>71</v>
       </c>
-      <c r="G4" s="24" t="s">
-        <v>15</v>
-      </c>
-      <c r="H4" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="I4" s="15" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" ht="36">
-      <c r="A5" s="12" t="s">
+      <c r="G4" s="22" t="s">
+        <v>15</v>
+      </c>
+      <c r="H4" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="I4" s="13" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="39.6" x14ac:dyDescent="0.3">
+      <c r="A5" s="10" t="s">
         <v>72</v>
       </c>
-      <c r="B5" s="12" t="s">
+      <c r="B5" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="C5" s="12" t="s">
+      <c r="C5" s="10" t="s">
         <v>74</v>
       </c>
-      <c r="D5" s="13" t="s">
+      <c r="D5" s="11" t="s">
         <v>75</v>
       </c>
-      <c r="E5" s="12" t="s">
+      <c r="E5" s="10" t="s">
         <v>76</v>
       </c>
-      <c r="F5" s="12" t="s">
+      <c r="F5" s="10" t="s">
         <v>77</v>
       </c>
-      <c r="G5" s="24" t="s">
-        <v>15</v>
-      </c>
-      <c r="H5" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="I5" s="15" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" ht="36">
-      <c r="A6" s="12" t="s">
+      <c r="G5" s="22" t="s">
+        <v>15</v>
+      </c>
+      <c r="H5" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="I5" s="13" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="39.6" x14ac:dyDescent="0.3">
+      <c r="A6" s="10" t="s">
         <v>78</v>
       </c>
-      <c r="B6" s="12" t="s">
+      <c r="B6" s="10" t="s">
         <v>79</v>
       </c>
-      <c r="C6" s="12" t="s">
+      <c r="C6" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="D6" s="13" t="s">
+      <c r="D6" s="11" t="s">
         <v>80</v>
       </c>
-      <c r="E6" s="12" t="s">
+      <c r="E6" s="10" t="s">
         <v>81</v>
       </c>
-      <c r="F6" s="12" t="s">
+      <c r="F6" s="10" t="s">
         <v>82</v>
       </c>
-      <c r="G6" s="24" t="s">
-        <v>15</v>
-      </c>
-      <c r="H6" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="I6" s="15" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" ht="36">
-      <c r="A7" s="12" t="s">
+      <c r="G6" s="22" t="s">
+        <v>15</v>
+      </c>
+      <c r="H6" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="I6" s="13" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="39.6" x14ac:dyDescent="0.3">
+      <c r="A7" s="10" t="s">
         <v>83</v>
       </c>
-      <c r="B7" s="12" t="s">
+      <c r="B7" s="10" t="s">
         <v>84</v>
       </c>
-      <c r="C7" s="12" t="s">
+      <c r="C7" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="D7" s="13" t="s">
+      <c r="D7" s="11" t="s">
         <v>85</v>
       </c>
-      <c r="E7" s="12" t="s">
+      <c r="E7" s="10" t="s">
         <v>86</v>
       </c>
-      <c r="F7" s="12" t="s">
+      <c r="F7" s="10" t="s">
         <v>87</v>
       </c>
-      <c r="G7" s="24" t="s">
-        <v>15</v>
-      </c>
-      <c r="H7" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="I7" s="15" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" ht="36">
-      <c r="A8" s="12" t="s">
+      <c r="G7" s="22" t="s">
+        <v>15</v>
+      </c>
+      <c r="H7" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="I7" s="13" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="39.6" x14ac:dyDescent="0.3">
+      <c r="A8" s="10" t="s">
         <v>88</v>
       </c>
-      <c r="B8" s="12" t="s">
+      <c r="B8" s="10" t="s">
         <v>89</v>
       </c>
-      <c r="C8" s="12" t="s">
+      <c r="C8" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="D8" s="13" t="s">
+      <c r="D8" s="11" t="s">
         <v>90</v>
       </c>
-      <c r="E8" s="12" t="s">
+      <c r="E8" s="10" t="s">
         <v>91</v>
       </c>
-      <c r="F8" s="12" t="s">
+      <c r="F8" s="10" t="s">
         <v>92</v>
       </c>
-      <c r="G8" s="24" t="s">
-        <v>15</v>
-      </c>
-      <c r="H8" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="I8" s="15" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" ht="39" customHeight="1">
-      <c r="A9" s="12" t="s">
+      <c r="G8" s="22" t="s">
+        <v>15</v>
+      </c>
+      <c r="H8" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="I8" s="13" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" ht="39" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="10" t="s">
         <v>93</v>
       </c>
-      <c r="B9" s="12" t="s">
+      <c r="B9" s="10" t="s">
         <v>94</v>
       </c>
-      <c r="C9" s="12" t="s">
+      <c r="C9" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="D9" s="13" t="s">
+      <c r="D9" s="11" t="s">
         <v>95</v>
       </c>
-      <c r="E9" s="12" t="s">
+      <c r="E9" s="10" t="s">
         <v>96</v>
       </c>
-      <c r="F9" s="12" t="s">
+      <c r="F9" s="10" t="s">
         <v>97</v>
       </c>
-      <c r="G9" s="25" t="s">
+      <c r="G9" s="23" t="s">
         <v>98</v>
       </c>
-      <c r="H9" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="I9" s="16" t="s">
+      <c r="H9" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="I9" s="14" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="33" customHeight="1">
-      <c r="A10" s="12" t="s">
+    <row r="10" spans="1:9" ht="33" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="10" t="s">
         <v>100</v>
       </c>
-      <c r="B10" s="12" t="s">
+      <c r="B10" s="10" t="s">
         <v>101</v>
       </c>
-      <c r="C10" s="12" t="s">
+      <c r="C10" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="D10" s="13" t="s">
+      <c r="D10" s="11" t="s">
         <v>102</v>
       </c>
-      <c r="E10" s="12">
+      <c r="E10" s="10">
         <v>-1</v>
       </c>
-      <c r="F10" s="12" t="s">
+      <c r="F10" s="10" t="s">
         <v>103</v>
       </c>
-      <c r="G10" s="25" t="s">
+      <c r="G10" s="23" t="s">
         <v>98</v>
       </c>
-      <c r="H10" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="I10" s="16" t="s">
+      <c r="H10" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="I10" s="14" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="24">
-      <c r="A11" s="12" t="s">
+    <row r="11" spans="1:9" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A11" s="10" t="s">
         <v>104</v>
       </c>
-      <c r="B11" s="12" t="s">
+      <c r="B11" s="10" t="s">
         <v>105</v>
       </c>
-      <c r="C11" s="12" t="s">
+      <c r="C11" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="D11" s="13" t="s">
+      <c r="D11" s="11" t="s">
         <v>106</v>
       </c>
-      <c r="E11" s="12" t="s">
+      <c r="E11" s="10" t="s">
         <v>107</v>
       </c>
-      <c r="F11" s="12" t="s">
+      <c r="F11" s="10" t="s">
         <v>108</v>
       </c>
-      <c r="G11" s="24" t="s">
-        <v>15</v>
-      </c>
-      <c r="H11" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="I11" s="17" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" ht="24">
-      <c r="A12" s="12" t="s">
+      <c r="G11" s="22" t="s">
+        <v>15</v>
+      </c>
+      <c r="H11" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="I11" s="15" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A12" s="10" t="s">
         <v>109</v>
       </c>
-      <c r="B12" s="12" t="s">
+      <c r="B12" s="10" t="s">
         <v>110</v>
       </c>
-      <c r="C12" s="12" t="s">
+      <c r="C12" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="D12" s="13" t="s">
+      <c r="D12" s="11" t="s">
         <v>111</v>
       </c>
-      <c r="E12" s="12" t="s">
+      <c r="E12" s="10" t="s">
         <v>112</v>
       </c>
-      <c r="F12" s="12" t="s">
+      <c r="F12" s="10" t="s">
         <v>108</v>
       </c>
-      <c r="G12" s="24" t="s">
-        <v>15</v>
-      </c>
-      <c r="H12" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="I12" s="17" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" ht="60">
-      <c r="A13" s="12" t="s">
+      <c r="G12" s="22" t="s">
+        <v>15</v>
+      </c>
+      <c r="H12" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="I12" s="15" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" ht="66" x14ac:dyDescent="0.3">
+      <c r="A13" s="10" t="s">
         <v>113</v>
       </c>
-      <c r="B13" s="19" t="s">
+      <c r="B13" s="17" t="s">
         <v>114</v>
       </c>
-      <c r="C13" s="18" t="s">
+      <c r="C13" s="16" t="s">
         <v>63</v>
       </c>
-      <c r="D13" s="20" t="s">
+      <c r="D13" s="18" t="s">
         <v>115</v>
       </c>
-      <c r="E13" s="21" t="s">
+      <c r="E13" s="19" t="s">
         <v>116</v>
       </c>
-      <c r="F13" s="22" t="s">
+      <c r="F13" s="20" t="s">
         <v>117</v>
       </c>
-      <c r="G13" s="19" t="s">
+      <c r="G13" s="17" t="s">
         <v>118</v>
       </c>
-      <c r="H13" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="I13" s="23" t="s">
+      <c r="H13" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="I13" s="21" t="s">
         <v>99</v>
       </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D61CACB2-AA2C-43C1-B0D6-67099275B8E2}">
-  <dimension ref="A1:H10"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="10.7109375" customWidth="1"/>
-    <col min="2" max="2" width="29.85546875" customWidth="1"/>
-    <col min="3" max="3" width="17" customWidth="1"/>
-    <col min="4" max="4" width="30.5703125" customWidth="1"/>
-    <col min="5" max="5" width="36.140625" customWidth="1"/>
-    <col min="7" max="7" width="14.42578125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:8" ht="28.5">
-      <c r="A1" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="5" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="F1" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="G1" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="H1" s="5" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" ht="24">
-      <c r="A2" s="6" t="s">
-        <v>119</v>
-      </c>
-      <c r="B2" s="9" t="s">
-        <v>120</v>
-      </c>
-      <c r="C2" s="9" t="s">
-        <v>121</v>
-      </c>
-      <c r="D2" s="10" t="s">
-        <v>122</v>
-      </c>
-      <c r="E2" s="9" t="s">
-        <v>123</v>
-      </c>
-      <c r="F2" s="1"/>
-      <c r="G2" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="H2" s="1"/>
-    </row>
-    <row r="3" spans="1:8" ht="24">
-      <c r="A3" s="6" t="s">
-        <v>124</v>
-      </c>
-      <c r="B3" s="9" t="s">
-        <v>125</v>
-      </c>
-      <c r="C3" s="9" t="s">
-        <v>126</v>
-      </c>
-      <c r="D3" s="10" t="s">
-        <v>127</v>
-      </c>
-      <c r="E3" s="9" t="s">
-        <v>128</v>
-      </c>
-      <c r="F3" s="1"/>
-      <c r="G3" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="H3" s="1"/>
-    </row>
-    <row r="4" spans="1:8" ht="36">
-      <c r="A4" s="6" t="s">
-        <v>129</v>
-      </c>
-      <c r="B4" s="9" t="s">
-        <v>130</v>
-      </c>
-      <c r="C4" s="9" t="s">
-        <v>126</v>
-      </c>
-      <c r="D4" s="10" t="s">
-        <v>131</v>
-      </c>
-      <c r="E4" s="9" t="s">
-        <v>132</v>
-      </c>
-      <c r="F4" s="1"/>
-      <c r="G4" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="H4" s="1"/>
-    </row>
-    <row r="5" spans="1:8" ht="48">
-      <c r="A5" s="6" t="s">
-        <v>133</v>
-      </c>
-      <c r="B5" s="9" t="s">
-        <v>134</v>
-      </c>
-      <c r="C5" s="9" t="s">
-        <v>126</v>
-      </c>
-      <c r="D5" s="10" t="s">
-        <v>135</v>
-      </c>
-      <c r="E5" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="F5" s="1"/>
-      <c r="G5" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="H5" s="1"/>
-    </row>
-    <row r="6" spans="1:8" ht="24">
-      <c r="A6" s="6" t="s">
-        <v>137</v>
-      </c>
-      <c r="B6" s="9" t="s">
-        <v>138</v>
-      </c>
-      <c r="C6" s="9" t="s">
-        <v>126</v>
-      </c>
-      <c r="D6" s="10" t="s">
-        <v>139</v>
-      </c>
-      <c r="E6" s="9" t="s">
-        <v>140</v>
-      </c>
-      <c r="F6" s="1"/>
-      <c r="G6" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="H6" s="1"/>
-    </row>
-    <row r="7" spans="1:8" ht="24">
-      <c r="A7" s="6" t="s">
-        <v>141</v>
-      </c>
-      <c r="B7" s="9" t="s">
-        <v>142</v>
-      </c>
-      <c r="C7" s="9" t="s">
-        <v>126</v>
-      </c>
-      <c r="D7" s="10" t="s">
-        <v>143</v>
-      </c>
-      <c r="E7" s="9" t="s">
-        <v>144</v>
-      </c>
-      <c r="F7" s="1"/>
-      <c r="G7" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="H7" s="1"/>
-    </row>
-    <row r="8" spans="1:8" ht="24">
-      <c r="A8" s="6" t="s">
-        <v>145</v>
-      </c>
-      <c r="B8" s="9" t="s">
-        <v>146</v>
-      </c>
-      <c r="C8" s="9" t="s">
-        <v>126</v>
-      </c>
-      <c r="D8" s="10" t="s">
-        <v>147</v>
-      </c>
-      <c r="E8" s="9" t="s">
-        <v>148</v>
-      </c>
-      <c r="F8" s="1"/>
-      <c r="G8" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="H8" s="1"/>
-    </row>
-    <row r="9" spans="1:8" ht="24">
-      <c r="A9" s="6" t="s">
-        <v>149</v>
-      </c>
-      <c r="B9" s="9" t="s">
-        <v>150</v>
-      </c>
-      <c r="C9" s="9" t="s">
-        <v>151</v>
-      </c>
-      <c r="D9" s="10" t="s">
-        <v>152</v>
-      </c>
-      <c r="E9" s="9" t="s">
-        <v>153</v>
-      </c>
-      <c r="F9" s="1"/>
-      <c r="G9" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="H9" s="1"/>
-    </row>
-    <row r="10" spans="1:8" ht="36">
-      <c r="A10" s="6" t="s">
-        <v>154</v>
-      </c>
-      <c r="B10" s="9" t="s">
-        <v>155</v>
-      </c>
-      <c r="C10" s="9" t="s">
-        <v>121</v>
-      </c>
-      <c r="D10" s="10" t="s">
-        <v>156</v>
-      </c>
-      <c r="E10" s="9" t="s">
-        <v>157</v>
-      </c>
-      <c r="F10" s="1"/>
-      <c r="G10" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="H10" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
sorting and filtering is done
</commit_message>
<xml_diff>
--- a/doc/coinmarketcap-test cases.xlsx
+++ b/doc/coinmarketcap-test cases.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30128"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{99CBA38C-4FBE-4D41-BF6D-1F2F71B932C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{70D64936-38BD-4CEE-9613-8841D802901E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="WF1 - Search" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="267" uniqueCount="158">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="277" uniqueCount="154">
   <si>
     <t>TC ID</t>
   </si>
@@ -472,7 +472,7 @@
     <t>TC_SF_04</t>
   </si>
   <si>
-    <t>Sort by Market Cap</t>
+    <t>Sort by Market Cap ascending</t>
   </si>
   <si>
     <t>1. Click the “Market Cap” column header
@@ -498,18 +498,6 @@
     <t>TC_SF_06</t>
   </si>
   <si>
-    <t>Jump to a specific page number</t>
-  </si>
-  <si>
-    <t>1. Click a specific page number (e.g. 3)</t>
-  </si>
-  <si>
-    <t>The table shows the coins belonging to that page</t>
-  </si>
-  <si>
-    <t>TC_SF_07</t>
-  </si>
-  <si>
     <t>Change rows per page</t>
   </si>
   <si>
@@ -520,7 +508,7 @@
     <t>The table displays the selected number of rows</t>
   </si>
   <si>
-    <t>TC_SF_08</t>
+    <t>TC_SF_07</t>
   </si>
   <si>
     <t>Pagination boundary on last page</t>
@@ -536,18 +524,18 @@
     <t>The “Next” control is disabled / no further page loads</t>
   </si>
   <si>
-    <t>TC_SF_09</t>
-  </si>
-  <si>
-    <t>Set layout to Top Gainers</t>
-  </si>
-  <si>
-    <t>1. Click Colums button
-2. Click on the drop down meun
-3. Select Top Gainers</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Coins are listed by rank (market cap), starting at 1, 2, 3 …
+    <t>TC_SF_08</t>
+  </si>
+  <si>
+    <t>Set filtring for the market cap</t>
+  </si>
+  <si>
+    <t>1. Click Filters button
+2. Set the min market cap = 100,000,000
+3. Set the max market cap = 150,000,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Coins are marketCap should be in this range
 </t>
   </si>
 </sst>
@@ -710,7 +698,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment readingOrder="1"/>
@@ -786,6 +774,9 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" readingOrder="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1812,7 +1803,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D61CACB2-AA2C-43C1-B0D6-67099275B8E2}">
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="10.7109375" customWidth="1"/>
@@ -1820,6 +1811,7 @@
     <col min="3" max="3" width="17" customWidth="1"/>
     <col min="4" max="4" width="30.5703125" customWidth="1"/>
     <col min="5" max="5" width="36.140625" customWidth="1"/>
+    <col min="6" max="6" width="12.5703125" customWidth="1"/>
     <col min="7" max="7" width="14.42578125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1865,11 +1857,15 @@
       <c r="E2" s="9" t="s">
         <v>123</v>
       </c>
-      <c r="F2" s="1"/>
+      <c r="F2" s="26" t="s">
+        <v>15</v>
+      </c>
       <c r="G2" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="H2" s="1"/>
+      <c r="H2" s="8" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="3" spans="1:8" ht="24">
       <c r="A3" s="6" t="s">
@@ -1887,11 +1883,15 @@
       <c r="E3" s="9" t="s">
         <v>128</v>
       </c>
-      <c r="F3" s="1"/>
+      <c r="F3" s="26" t="s">
+        <v>15</v>
+      </c>
       <c r="G3" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="H3" s="1"/>
+      <c r="H3" s="8" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="4" spans="1:8" ht="36">
       <c r="A4" s="6" t="s">
@@ -1909,11 +1909,15 @@
       <c r="E4" s="9" t="s">
         <v>132</v>
       </c>
-      <c r="F4" s="1"/>
+      <c r="F4" s="26" t="s">
+        <v>15</v>
+      </c>
       <c r="G4" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="H4" s="1"/>
+      <c r="H4" s="8" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="5" spans="1:8" ht="48">
       <c r="A5" s="6" t="s">
@@ -1931,11 +1935,15 @@
       <c r="E5" s="9" t="s">
         <v>136</v>
       </c>
-      <c r="F5" s="1"/>
+      <c r="F5" s="26" t="s">
+        <v>15</v>
+      </c>
       <c r="G5" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="H5" s="1"/>
+      <c r="H5" s="8" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="6" spans="1:8" ht="24">
       <c r="A6" s="6" t="s">
@@ -1953,11 +1961,15 @@
       <c r="E6" s="9" t="s">
         <v>140</v>
       </c>
-      <c r="F6" s="1"/>
+      <c r="F6" s="26" t="s">
+        <v>15</v>
+      </c>
       <c r="G6" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="H6" s="1"/>
+      <c r="H6" s="8" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="7" spans="1:8" ht="24">
       <c r="A7" s="6" t="s">
@@ -1975,11 +1987,15 @@
       <c r="E7" s="9" t="s">
         <v>144</v>
       </c>
-      <c r="F7" s="1"/>
+      <c r="F7" s="26" t="s">
+        <v>15</v>
+      </c>
       <c r="G7" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="H7" s="1"/>
+      <c r="H7" s="8" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="8" spans="1:8" ht="24">
       <c r="A8" s="6" t="s">
@@ -1989,29 +2005,33 @@
         <v>146</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>126</v>
+        <v>147</v>
       </c>
       <c r="D8" s="10" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>148</v>
-      </c>
-      <c r="F8" s="1"/>
+        <v>149</v>
+      </c>
+      <c r="F8" s="26" t="s">
+        <v>15</v>
+      </c>
       <c r="G8" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="H8" s="1"/>
-    </row>
-    <row r="9" spans="1:8" ht="24">
+      <c r="H8" s="8" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="60">
       <c r="A9" s="6" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="C9" s="9" t="s">
-        <v>151</v>
+        <v>121</v>
       </c>
       <c r="D9" s="10" t="s">
         <v>152</v>
@@ -2019,33 +2039,15 @@
       <c r="E9" s="9" t="s">
         <v>153</v>
       </c>
-      <c r="F9" s="1"/>
+      <c r="F9" s="26" t="s">
+        <v>15</v>
+      </c>
       <c r="G9" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="H9" s="1"/>
-    </row>
-    <row r="10" spans="1:8" ht="36">
-      <c r="A10" s="6" t="s">
-        <v>154</v>
-      </c>
-      <c r="B10" s="9" t="s">
-        <v>155</v>
-      </c>
-      <c r="C10" s="9" t="s">
-        <v>121</v>
-      </c>
-      <c r="D10" s="10" t="s">
-        <v>156</v>
-      </c>
-      <c r="E10" s="9" t="s">
-        <v>157</v>
-      </c>
-      <c r="F10" s="1"/>
-      <c r="G10" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="H10" s="1"/>
+      <c r="H9" s="8" t="s">
+        <v>17</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>